<commit_message>
Updated Sensitivity to 'Record' and validation for negative test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000186/negative/01/data/unit-test-CG0150-negative.xlsx
+++ b/rules/CORE-000186/negative/01/data/unit-test-CG0150-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -53,6 +53,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
@@ -65,7 +69,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -85,6 +89,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -108,14 +118,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,10 +469,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>3.4</v>
       </c>
     </row>
@@ -485,10 +496,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
@@ -501,7 +512,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -524,34 +535,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="C2" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>SUBJID</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>NotUnique1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="str">
         <v>dm.xpt</v>
       </c>
       <c r="C3" s="2" t="str">
-        <v>Variable</v>
+        <v>Record</v>
       </c>
       <c r="D3" s="2">
         <v>6</v>
@@ -563,9 +574,49 @@
         <v>NotUnique1</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>SUBJID</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>NotUnique2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="2">
+        <v>22</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>SUBJID</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>NotUnique2</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -643,1498 +694,1498 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Age</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Age Units</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Sex</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Race</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="5" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="5" t="str">
+      <c r="D3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="5" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="5" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="5" t="str">
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="5" t="str">
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="5" t="str">
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="K3" s="5" t="str">
+      <c r="K3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="L3" s="5" t="str">
+      <c r="L3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="M3" s="5" t="str">
+      <c r="M3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="N3" s="5" t="str">
+      <c r="N3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
+      <c r="O3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="P3" s="5" t="str">
+      <c r="P3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="Q3" s="5" t="str">
+      <c r="Q3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="R3" s="5" t="str">
+      <c r="R3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="S3" s="5" t="str">
+      <c r="S3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="T3" s="5" t="str">
+      <c r="T3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="U3" s="5" t="str">
+      <c r="U3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="V3" s="5" t="str">
+      <c r="V3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>14</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>10</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>10</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>10</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>10</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>10</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>10</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>1</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>1</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>3</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>5</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>1</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>1</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="6">
         <v>1</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="6">
         <v>13</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="6">
         <v>1</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="6">
         <v>13</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC-TEST-001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="7" t="str">
         <v>NotUnique1</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>2019-03-12</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>2019-09-10</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>2019-03-12</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>2019-09-10</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>2019-02-25</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>2019-10-10</v>
       </c>
-      <c r="K5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M5" s="6" t="str">
+      <c r="K5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M5" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="4">
         <v>26</v>
       </c>
-      <c r="O5" s="6" t="str">
+      <c r="O5" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R5" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S5" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T5" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U5" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V5" s="6" t="str">
+      <c r="Q5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R5" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S5" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T5" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U5" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V5" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC-TEST-002</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="7" t="str">
         <v>NotUnique1</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>2019-01-30</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>2019-07-31</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>2019-01-30</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>2019-07-31</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>2019-01-15</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="4" t="str">
         <v>2019-08-30</v>
       </c>
-      <c r="K6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M6" s="6" t="str">
+      <c r="K6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M6" s="4" t="str">
         <v>103</v>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="4">
         <v>34</v>
       </c>
-      <c r="O6" s="6" t="str">
+      <c r="O6" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P6" s="6" t="str">
+      <c r="P6" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R6" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S6" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T6" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U6" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V6" s="6" t="str">
+      <c r="Q6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R6" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S6" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T6" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U6" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V6" s="4" t="str">
         <v>JPN</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC-TEST-003</v>
       </c>
-      <c r="D7" s="6" t="str">
+      <c r="D7" s="4" t="str">
         <v>003</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="4" t="str">
         <v>2019-01-26</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="4" t="str">
         <v>2019-07-27</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>2019-01-26</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>2019-07-27</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>2019-01-11</v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="4" t="str">
         <v>2019-08-26</v>
       </c>
-      <c r="K7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M7" s="6" t="str">
+      <c r="K7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M7" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="4">
         <v>57</v>
       </c>
-      <c r="O7" s="6" t="str">
+      <c r="O7" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P7" s="6" t="str">
+      <c r="P7" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R7" s="6" t="str">
+      <c r="Q7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R7" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S7" s="6" t="str">
+      <c r="S7" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T7" s="6" t="str">
+      <c r="T7" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U7" s="6" t="str">
+      <c r="U7" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V7" s="6" t="str">
+      <c r="V7" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC-TEST-004</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="4" t="str">
         <v>004</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>2019-02-16</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>2019-08-17</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="4" t="str">
         <v>2019-02-16</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>2019-08-17</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="4" t="str">
         <v>2019-02-01</v>
       </c>
-      <c r="J8" s="6" t="str">
+      <c r="J8" s="4" t="str">
         <v>2019-09-16</v>
       </c>
-      <c r="K8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M8" s="6" t="str">
+      <c r="K8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M8" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="4">
         <v>31</v>
       </c>
-      <c r="O8" s="6" t="str">
+      <c r="O8" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P8" s="6" t="str">
+      <c r="P8" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R8" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S8" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T8" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U8" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V8" s="6" t="str">
+      <c r="Q8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R8" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S8" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T8" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U8" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V8" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B9" s="6" t="str">
+      <c r="B9" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC-TEST-005</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="4" t="str">
         <v>005</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E9" s="4" t="str">
         <v>2019-03-02</v>
       </c>
-      <c r="F9" s="6" t="str">
+      <c r="F9" s="4" t="str">
         <v>2019-08-31</v>
       </c>
-      <c r="G9" s="6" t="str">
+      <c r="G9" s="4" t="str">
         <v>2019-03-02</v>
       </c>
-      <c r="H9" s="6" t="str">
+      <c r="H9" s="4" t="str">
         <v>2019-08-31</v>
       </c>
-      <c r="I9" s="6" t="str">
+      <c r="I9" s="4" t="str">
         <v>2019-02-15</v>
       </c>
-      <c r="J9" s="6" t="str">
+      <c r="J9" s="4" t="str">
         <v>2019-09-30</v>
       </c>
-      <c r="K9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M9" s="6" t="str">
+      <c r="K9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M9" s="4" t="str">
         <v>103</v>
       </c>
-      <c r="N9" s="6">
+      <c r="N9" s="4">
         <v>21</v>
       </c>
-      <c r="O9" s="6" t="str">
+      <c r="O9" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P9" s="6" t="str">
+      <c r="P9" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R9" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S9" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T9" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U9" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V9" s="6" t="str">
+      <c r="Q9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R9" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S9" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T9" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U9" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V9" s="4" t="str">
         <v>JPN</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="str">
+      <c r="A10" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B10" s="6" t="str">
+      <c r="B10" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC-TEST-006</v>
       </c>
-      <c r="D10" s="6" t="str">
+      <c r="D10" s="4" t="str">
         <v>006</v>
       </c>
-      <c r="E10" s="6" t="str">
+      <c r="E10" s="4" t="str">
         <v>2019-02-18</v>
       </c>
-      <c r="F10" s="6" t="str">
+      <c r="F10" s="4" t="str">
         <v>2019-08-19</v>
       </c>
-      <c r="G10" s="6" t="str">
+      <c r="G10" s="4" t="str">
         <v>2019-02-18</v>
       </c>
-      <c r="H10" s="6" t="str">
+      <c r="H10" s="4" t="str">
         <v>2019-08-19</v>
       </c>
-      <c r="I10" s="6" t="str">
+      <c r="I10" s="4" t="str">
         <v>2019-02-03</v>
       </c>
-      <c r="J10" s="6" t="str">
+      <c r="J10" s="4" t="str">
         <v>2019-09-18</v>
       </c>
-      <c r="K10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M10" s="6" t="str">
+      <c r="K10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M10" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N10" s="6">
+      <c r="N10" s="4">
         <v>52</v>
       </c>
-      <c r="O10" s="6" t="str">
+      <c r="O10" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P10" s="6" t="str">
+      <c r="P10" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R10" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S10" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T10" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U10" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V10" s="6" t="str">
+      <c r="Q10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R10" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S10" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T10" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U10" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V10" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B11" s="6" t="str">
+      <c r="B11" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC-TEST-007</v>
       </c>
-      <c r="D11" s="6" t="str">
+      <c r="D11" s="4" t="str">
         <v>007</v>
       </c>
-      <c r="E11" s="6" t="str">
+      <c r="E11" s="4" t="str">
         <v>2019-02-25</v>
       </c>
-      <c r="F11" s="6" t="str">
+      <c r="F11" s="4" t="str">
         <v>2019-08-26</v>
       </c>
-      <c r="G11" s="6" t="str">
+      <c r="G11" s="4" t="str">
         <v>2019-02-25</v>
       </c>
-      <c r="H11" s="6" t="str">
+      <c r="H11" s="4" t="str">
         <v>2019-08-26</v>
       </c>
-      <c r="I11" s="6" t="str">
+      <c r="I11" s="4" t="str">
         <v>2019-02-10</v>
       </c>
-      <c r="J11" s="6" t="str">
+      <c r="J11" s="4" t="str">
         <v>2019-09-25</v>
       </c>
-      <c r="K11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M11" s="6" t="str">
+      <c r="K11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M11" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N11" s="4">
         <v>57</v>
       </c>
-      <c r="O11" s="6" t="str">
+      <c r="O11" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P11" s="6" t="str">
+      <c r="P11" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R11" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S11" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T11" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U11" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V11" s="6" t="str">
+      <c r="Q11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R11" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S11" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T11" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U11" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V11" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="str">
+      <c r="A12" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B12" s="6" t="str">
+      <c r="B12" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC-TEST-008</v>
       </c>
-      <c r="D12" s="6" t="str">
+      <c r="D12" s="4" t="str">
         <v>008</v>
       </c>
-      <c r="E12" s="6" t="str">
+      <c r="E12" s="4" t="str">
         <v>2019-02-06</v>
       </c>
-      <c r="F12" s="6" t="str">
+      <c r="F12" s="4" t="str">
         <v>2019-08-07</v>
       </c>
-      <c r="G12" s="6" t="str">
+      <c r="G12" s="4" t="str">
         <v>2019-02-06</v>
       </c>
-      <c r="H12" s="6" t="str">
+      <c r="H12" s="4" t="str">
         <v>2019-08-07</v>
       </c>
-      <c r="I12" s="6" t="str">
+      <c r="I12" s="4" t="str">
         <v>2019-01-22</v>
       </c>
-      <c r="J12" s="6" t="str">
+      <c r="J12" s="4" t="str">
         <v>2019-09-06</v>
       </c>
-      <c r="K12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M12" s="6" t="str">
+      <c r="K12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M12" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N12" s="6">
+      <c r="N12" s="4">
         <v>50</v>
       </c>
-      <c r="O12" s="6" t="str">
+      <c r="O12" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P12" s="6" t="str">
+      <c r="P12" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R12" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S12" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T12" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U12" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V12" s="6" t="str">
+      <c r="Q12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R12" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S12" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T12" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U12" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V12" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="str">
+      <c r="A13" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B13" s="6" t="str">
+      <c r="B13" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C13" s="6" t="str">
+      <c r="C13" s="4" t="str">
         <v>CDISC-TEST-009</v>
       </c>
-      <c r="D13" s="6" t="str">
+      <c r="D13" s="4" t="str">
         <v>009</v>
       </c>
-      <c r="E13" s="6" t="str">
+      <c r="E13" s="4" t="str">
         <v>2019-01-25</v>
       </c>
-      <c r="F13" s="6" t="str">
+      <c r="F13" s="4" t="str">
         <v>2019-07-26</v>
       </c>
-      <c r="G13" s="6" t="str">
+      <c r="G13" s="4" t="str">
         <v>2019-01-25</v>
       </c>
-      <c r="H13" s="6" t="str">
+      <c r="H13" s="4" t="str">
         <v>2019-07-26</v>
       </c>
-      <c r="I13" s="6" t="str">
+      <c r="I13" s="4" t="str">
         <v>2019-01-10</v>
       </c>
-      <c r="J13" s="6" t="str">
+      <c r="J13" s="4" t="str">
         <v>2019-08-25</v>
       </c>
-      <c r="K13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M13" s="6" t="str">
+      <c r="K13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M13" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N13" s="6">
+      <c r="N13" s="4">
         <v>48</v>
       </c>
-      <c r="O13" s="6" t="str">
+      <c r="O13" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P13" s="6" t="str">
+      <c r="P13" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R13" s="6" t="str">
+      <c r="Q13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R13" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S13" s="6" t="str">
+      <c r="S13" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T13" s="6" t="str">
+      <c r="T13" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U13" s="6" t="str">
+      <c r="U13" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V13" s="6" t="str">
+      <c r="V13" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="str">
+      <c r="A14" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B14" s="6" t="str">
+      <c r="B14" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC-TEST-010</v>
       </c>
-      <c r="D14" s="6" t="str">
+      <c r="D14" s="4" t="str">
         <v>010</v>
       </c>
-      <c r="E14" s="6" t="str">
+      <c r="E14" s="4" t="str">
         <v>2019-01-22</v>
       </c>
-      <c r="F14" s="6" t="str">
+      <c r="F14" s="4" t="str">
         <v>2019-07-23</v>
       </c>
-      <c r="G14" s="6" t="str">
+      <c r="G14" s="4" t="str">
         <v>2019-01-22</v>
       </c>
-      <c r="H14" s="6" t="str">
+      <c r="H14" s="4" t="str">
         <v>2019-07-23</v>
       </c>
-      <c r="I14" s="6" t="str">
+      <c r="I14" s="4" t="str">
         <v>2019-01-07</v>
       </c>
-      <c r="J14" s="6" t="str">
+      <c r="J14" s="4" t="str">
         <v>2019-08-22</v>
       </c>
-      <c r="K14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M14" s="6" t="str">
+      <c r="K14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M14" s="4" t="str">
         <v>103</v>
       </c>
-      <c r="N14" s="6">
+      <c r="N14" s="4">
         <v>32</v>
       </c>
-      <c r="O14" s="6" t="str">
+      <c r="O14" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P14" s="6" t="str">
+      <c r="P14" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R14" s="6" t="str">
+      <c r="Q14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R14" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S14" s="6" t="str">
+      <c r="S14" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T14" s="6" t="str">
+      <c r="T14" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U14" s="6" t="str">
+      <c r="U14" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V14" s="6" t="str">
+      <c r="V14" s="4" t="str">
         <v>JPN</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="str">
+      <c r="A15" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B15" s="6" t="str">
+      <c r="B15" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C15" s="6" t="str">
+      <c r="C15" s="4" t="str">
         <v>CDISC-TEST-011</v>
       </c>
-      <c r="D15" s="6" t="str">
+      <c r="D15" s="4" t="str">
         <v>011</v>
       </c>
-      <c r="E15" s="6" t="str">
+      <c r="E15" s="4" t="str">
         <v>2019-02-10</v>
       </c>
-      <c r="F15" s="6" t="str">
+      <c r="F15" s="4" t="str">
         <v>2019-08-11</v>
       </c>
-      <c r="G15" s="6" t="str">
+      <c r="G15" s="4" t="str">
         <v>2019-02-10</v>
       </c>
-      <c r="H15" s="6" t="str">
+      <c r="H15" s="4" t="str">
         <v>2019-08-11</v>
       </c>
-      <c r="I15" s="6" t="str">
+      <c r="I15" s="4" t="str">
         <v>2019-01-26</v>
       </c>
-      <c r="J15" s="6" t="str">
+      <c r="J15" s="4" t="str">
         <v>2019-09-10</v>
       </c>
-      <c r="K15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M15" s="6" t="str">
+      <c r="K15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M15" s="4" t="str">
         <v>101</v>
       </c>
-      <c r="N15" s="6">
+      <c r="N15" s="4">
         <v>63</v>
       </c>
-      <c r="O15" s="6" t="str">
+      <c r="O15" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P15" s="6" t="str">
+      <c r="P15" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R15" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S15" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T15" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U15" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V15" s="6" t="str">
+      <c r="Q15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R15" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S15" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T15" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U15" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V15" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="str">
+      <c r="A16" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B16" s="6" t="str">
+      <c r="B16" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C16" s="6" t="str">
+      <c r="C16" s="4" t="str">
         <v>CDISC-TEST-012</v>
       </c>
-      <c r="D16" s="6" t="str">
+      <c r="D16" s="4" t="str">
         <v>012</v>
       </c>
-      <c r="E16" s="6" t="str">
+      <c r="E16" s="4" t="str">
         <v>2019-03-15</v>
       </c>
-      <c r="F16" s="6" t="str">
+      <c r="F16" s="4" t="str">
         <v>2019-09-13</v>
       </c>
-      <c r="G16" s="6" t="str">
+      <c r="G16" s="4" t="str">
         <v>2019-03-15</v>
       </c>
-      <c r="H16" s="6" t="str">
+      <c r="H16" s="4" t="str">
         <v>2019-09-13</v>
       </c>
-      <c r="I16" s="6" t="str">
+      <c r="I16" s="4" t="str">
         <v>2019-02-28</v>
       </c>
-      <c r="J16" s="6" t="str">
+      <c r="J16" s="4" t="str">
         <v>2019-10-13</v>
       </c>
-      <c r="K16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M16" s="6" t="str">
+      <c r="K16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M16" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N16" s="6">
+      <c r="N16" s="4">
         <v>57</v>
       </c>
-      <c r="O16" s="6" t="str">
+      <c r="O16" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P16" s="6" t="str">
+      <c r="P16" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R16" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S16" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T16" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U16" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V16" s="6" t="str">
+      <c r="Q16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R16" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S16" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T16" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U16" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V16" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="str">
+      <c r="A17" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B17" s="6" t="str">
+      <c r="B17" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C17" s="6" t="str">
+      <c r="C17" s="4" t="str">
         <v>CDISC-TEST-013</v>
       </c>
-      <c r="D17" s="6" t="str">
+      <c r="D17" s="4" t="str">
         <v>013</v>
       </c>
-      <c r="E17" s="6" t="str">
+      <c r="E17" s="4" t="str">
         <v>2019-03-10</v>
       </c>
-      <c r="F17" s="6" t="str">
+      <c r="F17" s="4" t="str">
         <v>2019-09-08</v>
       </c>
-      <c r="G17" s="6" t="str">
+      <c r="G17" s="4" t="str">
         <v>2019-03-10</v>
       </c>
-      <c r="H17" s="6" t="str">
+      <c r="H17" s="4" t="str">
         <v>2019-09-08</v>
       </c>
-      <c r="I17" s="6" t="str">
+      <c r="I17" s="4" t="str">
         <v>2019-02-23</v>
       </c>
-      <c r="J17" s="6" t="str">
+      <c r="J17" s="4" t="str">
         <v>2019-10-08</v>
       </c>
-      <c r="K17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M17" s="6" t="str">
+      <c r="K17" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L17" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M17" s="4" t="str">
         <v>103</v>
       </c>
-      <c r="N17" s="6">
+      <c r="N17" s="4">
         <v>31</v>
       </c>
-      <c r="O17" s="6" t="str">
+      <c r="O17" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P17" s="6" t="str">
+      <c r="P17" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R17" s="6" t="str">
+      <c r="Q17" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R17" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S17" s="6" t="str">
+      <c r="S17" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T17" s="6" t="str">
+      <c r="T17" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U17" s="6" t="str">
+      <c r="U17" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V17" s="6" t="str">
+      <c r="V17" s="4" t="str">
         <v>JPN</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="str">
+      <c r="A18" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B18" s="6" t="str">
+      <c r="B18" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C18" s="6" t="str">
+      <c r="C18" s="4" t="str">
         <v>CDISC-TEST-014</v>
       </c>
-      <c r="D18" s="6" t="str">
+      <c r="D18" s="4" t="str">
         <v>014</v>
       </c>
-      <c r="E18" s="6" t="str">
+      <c r="E18" s="4" t="str">
         <v>2019-02-18</v>
       </c>
-      <c r="F18" s="6" t="str">
+      <c r="F18" s="4" t="str">
         <v>2019-08-19</v>
       </c>
-      <c r="G18" s="6" t="str">
+      <c r="G18" s="4" t="str">
         <v>2019-02-18</v>
       </c>
-      <c r="H18" s="6" t="str">
+      <c r="H18" s="4" t="str">
         <v>2019-08-19</v>
       </c>
-      <c r="I18" s="6" t="str">
+      <c r="I18" s="4" t="str">
         <v>2019-02-03</v>
       </c>
-      <c r="J18" s="6" t="str">
+      <c r="J18" s="4" t="str">
         <v>2019-09-18</v>
       </c>
-      <c r="K18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M18" s="6" t="str">
+      <c r="K18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M18" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N18" s="6">
+      <c r="N18" s="4">
         <v>56</v>
       </c>
-      <c r="O18" s="6" t="str">
+      <c r="O18" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P18" s="6" t="str">
+      <c r="P18" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R18" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S18" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T18" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U18" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V18" s="6" t="str">
+      <c r="Q18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R18" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S18" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T18" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U18" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V18" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="str">
+      <c r="A19" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B19" s="6" t="str">
+      <c r="B19" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C19" s="6" t="str">
+      <c r="C19" s="4" t="str">
         <v>CDISC-TEST-015</v>
       </c>
-      <c r="D19" s="6" t="str">
+      <c r="D19" s="4" t="str">
         <v>015</v>
       </c>
-      <c r="E19" s="6" t="str">
+      <c r="E19" s="4" t="str">
         <v>2019-01-29</v>
       </c>
-      <c r="F19" s="6" t="str">
+      <c r="F19" s="4" t="str">
         <v>2019-07-30</v>
       </c>
-      <c r="G19" s="6" t="str">
+      <c r="G19" s="4" t="str">
         <v>2019-01-29</v>
       </c>
-      <c r="H19" s="6" t="str">
+      <c r="H19" s="4" t="str">
         <v>2019-07-30</v>
       </c>
-      <c r="I19" s="6" t="str">
+      <c r="I19" s="4" t="str">
         <v>2019-01-14</v>
       </c>
-      <c r="J19" s="6" t="str">
+      <c r="J19" s="4" t="str">
         <v>2019-08-29</v>
       </c>
-      <c r="K19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M19" s="6" t="str">
+      <c r="K19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M19" s="4" t="str">
         <v>101</v>
       </c>
-      <c r="N19" s="6">
+      <c r="N19" s="4">
         <v>21</v>
       </c>
-      <c r="O19" s="6" t="str">
+      <c r="O19" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P19" s="6" t="str">
+      <c r="P19" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R19" s="6" t="str">
+      <c r="Q19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R19" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S19" s="6" t="str">
+      <c r="S19" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T19" s="6" t="str">
+      <c r="T19" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U19" s="6" t="str">
+      <c r="U19" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V19" s="6" t="str">
+      <c r="V19" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="str">
+      <c r="A20" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B20" s="6" t="str">
+      <c r="B20" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C20" s="6" t="str">
+      <c r="C20" s="4" t="str">
         <v>CDISC-TEST-016</v>
       </c>
-      <c r="D20" s="6" t="str">
+      <c r="D20" s="4" t="str">
         <v>016</v>
       </c>
-      <c r="E20" s="6" t="str">
+      <c r="E20" s="4" t="str">
         <v>2019-03-02</v>
       </c>
-      <c r="F20" s="6" t="str">
+      <c r="F20" s="4" t="str">
         <v>2019-08-31</v>
       </c>
-      <c r="G20" s="6" t="str">
+      <c r="G20" s="4" t="str">
         <v>2019-03-02</v>
       </c>
-      <c r="H20" s="6" t="str">
+      <c r="H20" s="4" t="str">
         <v>2019-08-31</v>
       </c>
-      <c r="I20" s="6" t="str">
+      <c r="I20" s="4" t="str">
         <v>2019-02-15</v>
       </c>
-      <c r="J20" s="6" t="str">
+      <c r="J20" s="4" t="str">
         <v>2019-09-30</v>
       </c>
-      <c r="K20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M20" s="6" t="str">
+      <c r="K20" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L20" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M20" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N20" s="6">
+      <c r="N20" s="4">
         <v>51</v>
       </c>
-      <c r="O20" s="6" t="str">
+      <c r="O20" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P20" s="6" t="str">
+      <c r="P20" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R20" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S20" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T20" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U20" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V20" s="6" t="str">
+      <c r="Q20" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R20" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S20" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T20" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U20" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V20" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="str">
+      <c r="A21" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B21" s="6" t="str">
+      <c r="B21" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C21" s="6" t="str">
+      <c r="C21" s="4" t="str">
         <v>CDISC-TEST-017</v>
       </c>
-      <c r="D21" s="6" t="str">
-        <v>017</v>
-      </c>
-      <c r="E21" s="6" t="str">
+      <c r="D21" s="7" t="str">
+        <v>NotUnique2</v>
+      </c>
+      <c r="E21" s="4" t="str">
         <v>2019-02-09</v>
       </c>
-      <c r="F21" s="6" t="str">
+      <c r="F21" s="4" t="str">
         <v>2019-08-10</v>
       </c>
-      <c r="G21" s="6" t="str">
+      <c r="G21" s="4" t="str">
         <v>2019-02-09</v>
       </c>
-      <c r="H21" s="6" t="str">
+      <c r="H21" s="4" t="str">
         <v>2019-08-10</v>
       </c>
-      <c r="I21" s="6" t="str">
+      <c r="I21" s="4" t="str">
         <v>2019-01-25</v>
       </c>
-      <c r="J21" s="6" t="str">
+      <c r="J21" s="4" t="str">
         <v>2019-09-09</v>
       </c>
-      <c r="K21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M21" s="6" t="str">
+      <c r="K21" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L21" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M21" s="4" t="str">
         <v>102</v>
       </c>
-      <c r="N21" s="6">
+      <c r="N21" s="4">
         <v>48</v>
       </c>
-      <c r="O21" s="6" t="str">
+      <c r="O21" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P21" s="6" t="str">
+      <c r="P21" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R21" s="6" t="str">
+      <c r="Q21" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R21" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S21" s="6" t="str">
+      <c r="S21" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T21" s="6" t="str">
+      <c r="T21" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U21" s="6" t="str">
+      <c r="U21" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V21" s="6" t="str">
+      <c r="V21" s="4" t="str">
         <v>FRA</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="str">
+      <c r="A22" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B22" s="6" t="str">
+      <c r="B22" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C22" s="6" t="str">
+      <c r="C22" s="4" t="str">
         <v>CDISC-TEST-019</v>
       </c>
-      <c r="D22" s="6">
-        <v>18</v>
-      </c>
-      <c r="E22" s="6" t="str">
+      <c r="D22" s="7" t="str">
+        <v>NotUnique2</v>
+      </c>
+      <c r="E22" s="4" t="str">
         <v>2019-03-07</v>
       </c>
-      <c r="F22" s="6" t="str">
+      <c r="F22" s="4" t="str">
         <v>2019-09-05</v>
       </c>
-      <c r="G22" s="6" t="str">
+      <c r="G22" s="4" t="str">
         <v>2019-03-07</v>
       </c>
-      <c r="H22" s="6" t="str">
+      <c r="H22" s="4" t="str">
         <v>2019-09-05</v>
       </c>
-      <c r="I22" s="6" t="str">
+      <c r="I22" s="4" t="str">
         <v>2019-02-20</v>
       </c>
-      <c r="J22" s="6" t="str">
+      <c r="J22" s="4" t="str">
         <v>2019-10-05</v>
       </c>
-      <c r="K22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M22" s="6" t="str">
+      <c r="K22" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L22" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M22" s="4" t="str">
         <v>101</v>
       </c>
-      <c r="N22" s="6">
+      <c r="N22" s="4">
         <v>19</v>
       </c>
-      <c r="O22" s="6" t="str">
+      <c r="O22" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P22" s="6" t="str">
+      <c r="P22" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="Q22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R22" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="S22" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="T22" s="6" t="str">
-        <v>A</v>
-      </c>
-      <c r="U22" s="6" t="str">
-        <v>HUMAN INSULIN</v>
-      </c>
-      <c r="V22" s="6" t="str">
+      <c r="Q22" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R22" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="S22" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="T22" s="4" t="str">
+        <v>A</v>
+      </c>
+      <c r="U22" s="4" t="str">
+        <v>HUMAN INSULIN</v>
+      </c>
+      <c r="V22" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="str">
+      <c r="A23" s="4" t="str">
         <v>CDISC-TEST</v>
       </c>
-      <c r="B23" s="6" t="str">
+      <c r="B23" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C23" s="6" t="str">
+      <c r="C23" s="4" t="str">
         <v>CDISC-TEST-020</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="4">
         <v>19</v>
       </c>
-      <c r="E23" s="6" t="str">
+      <c r="E23" s="4" t="str">
         <v>2019-01-18</v>
       </c>
-      <c r="F23" s="6" t="str">
+      <c r="F23" s="4" t="str">
         <v>2019-07-19</v>
       </c>
-      <c r="G23" s="6" t="str">
+      <c r="G23" s="4" t="str">
         <v>2019-01-18</v>
       </c>
-      <c r="H23" s="6" t="str">
+      <c r="H23" s="4" t="str">
         <v>2019-07-19</v>
       </c>
-      <c r="I23" s="6" t="str">
+      <c r="I23" s="4" t="str">
         <v>2019-01-03</v>
       </c>
-      <c r="J23" s="6" t="str">
+      <c r="J23" s="4" t="str">
         <v>2019-08-18</v>
       </c>
-      <c r="K23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M23" s="6" t="str">
+      <c r="K23" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L23" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M23" s="4" t="str">
         <v>103</v>
       </c>
-      <c r="N23" s="6">
+      <c r="N23" s="4">
         <v>33</v>
       </c>
-      <c r="O23" s="6" t="str">
+      <c r="O23" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="P23" s="6" t="str">
+      <c r="P23" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="Q23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="R23" s="6" t="str">
+      <c r="Q23" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R23" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="S23" s="6" t="str">
+      <c r="S23" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="T23" s="6" t="str">
+      <c r="T23" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="U23" s="6" t="str">
+      <c r="U23" s="4" t="str">
         <v>METFORMIN</v>
       </c>
-      <c r="V23" s="6" t="str">
+      <c r="V23" s="4" t="str">
         <v>JPN</v>
       </c>
     </row>

</xml_diff>